<commit_message>
Add hero style variant and updated dell importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (9):
- blocks/hero/hero.css
- blocks/hero/hero.js
- styles/styles.css
- tools/importer/import-pc-landing-page.bundle.js
- tools/importer/import-pc-landing-page.js
- tools/importer/reports/en-us/lp/aipc.report.json
- tools/importer/reports/en-us/lp/dell-pro-max-pcs.report.json
- tools/importer/reports/import-pc-landing-page.report.xlsx
- tools/importer/transformers/dell-cleanup.js
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-pc-landing-page.report.xlsx
+++ b/tools/importer/reports/import-pc-landing-page.report.xlsx
@@ -61,7 +61,7 @@
     <t>pc-landing-page</t>
   </si>
   <si>
-    <t>2026-03-23T16:26:13.306Z</t>
+    <t>2026-03-23T16:51:16.965Z</t>
   </si>
   <si>
     <t>Dell AI Laptops &amp; PCs with Intel Processors | Dell USA</t>
@@ -100,7 +100,7 @@
     <t>en-us/lp/dell-pro-max-pcs</t>
   </si>
   <si>
-    <t>2026-03-23T16:26:20.875Z</t>
+    <t>2026-03-23T16:51:23.302Z</t>
   </si>
   <si>
     <t>Dell Pro Max High-Performance PCs, Laptops &amp; Desktops | Dell USA</t>

</xml_diff>

<commit_message>
Add agreements, cards, showcase blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (13):
- blocks/agreements/agreements.css
- blocks/agreements/agreements.js
- blocks/cards/cards.css
- blocks/showcase/showcase.css
- blocks/showcase/showcase.js
- tools/importer/import-pc-landing-page.bundle.js
- tools/importer/import-pc-landing-page.js
- tools/importer/parsers/agreements.js
- tools/importer/parsers/showcase.js
- tools/importer/reports/en-us/lp/aipc.report.json
- tools/importer/reports/en-us/lp/dell-pro-max-pcs.report.json
- tools/importer/reports/import-pc-landing-page.report.xlsx
- tools/importer/transformers/dell-cleanup.js
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-pc-landing-page.report.xlsx
+++ b/tools/importer/reports/import-pc-landing-page.report.xlsx
@@ -46,7 +46,7 @@
     <t>en-us/lp/aipc.report.json</t>
   </si>
   <si>
-    <t>["hero","hero","hero","hero","hero","columns","columns","cards","cards","cards","cards","cards","cards","accordion","accordion"]</t>
+    <t>["agreements","agreements","hero","hero","hero","hero","hero","columns","columns","cards","cards","cards","cards","cards","cards","accordion","accordion"]</t>
   </si>
   <si>
     <t/>
@@ -61,7 +61,7 @@
     <t>pc-landing-page</t>
   </si>
   <si>
-    <t>2026-03-23T16:51:16.965Z</t>
+    <t>2026-03-24T15:54:14.087Z</t>
   </si>
   <si>
     <t>Dell AI Laptops &amp; PCs with Intel Processors | Dell USA</t>
@@ -94,13 +94,13 @@
     <t>en-us/lp/dell-pro-max-pcs.report.json</t>
   </si>
   <si>
-    <t>["hero","columns","columns","cards","cards","accordion"]</t>
+    <t>["agreements","agreements","hero","showcase","showcase","showcase","columns","columns","cards","cards","accordion"]</t>
   </si>
   <si>
     <t>en-us/lp/dell-pro-max-pcs</t>
   </si>
   <si>
-    <t>2026-03-23T16:51:23.302Z</t>
+    <t>2026-03-24T15:54:22.184Z</t>
   </si>
   <si>
     <t>Dell Pro Max High-Performance PCs, Laptops &amp; Desktops | Dell USA</t>

</xml_diff>